<commit_message>
feat: implement modular GUI architecture with dedicated frames for student, academic, and administrative modules.
</commit_message>
<xml_diff>
--- a/assets/templates/Registro_Primaria.xlsx
+++ b/assets/templates/Registro_Primaria.xlsx
@@ -2517,7 +2517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A7:BQ54"/>
+  <dimension ref="A7:AD25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="147" min="1" max="39"/>
@@ -2554,10 +2554,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23" ht="17.4" customHeight="1" s="147">
       <c r="Q23" s="172" t="n"/>
     </row>
@@ -2567,35 +2563,6 @@
     <row r="25" ht="17.4" customHeight="1" s="147">
       <c r="Q25" s="172" t="n"/>
     </row>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="L7:T7"/>

</xml_diff>